<commit_message>
feat(F-NAR-019): TREE-AUT-023 polish Le manteau sur la rampe
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-023.xlsx
+++ b/stories/arbres/TREE-AUT-023.xlsx
@@ -2748,17 +2748,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le grain a failli tout cacher. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Un grain cachait le croissant, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le grain a failli tout cacher. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Un grain cachait le croissant, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le grain a failli tout cacher. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Un grain cachait le croissant, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2915,7 +2915,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Un grain de sable reste au croissant.
-narrateur|Le grain a failli tout cacher.
+narrateur|Un grain cachait le croissant, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -3139,17 +3139,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le loquet a failli tout garder. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le loquet serrait trop, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le loquet a failli tout garder. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le loquet serrait trop, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le loquet a failli tout garder. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. Le loquet serrait trop, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Un grain de sable reste au croissant.
-narrateur|Le loquet a failli tout garder.
+narrateur|Le loquet serrait trop, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -3339,17 +3339,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Le couloir sent les fraises, plus fort. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le loquet garde un fil rouge.</t>
+          <t>Le couloir sent les fraises, plus fort. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le loquet garde un fil rouge, minuscule.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couloir sent les fraises, plus fort. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le loquet garde un fil rouge.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couloir sent les fraises, plus fort. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le loquet garde un fil rouge, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couloir sent les fraises, plus fort. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le loquet garde un fil rouge.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couloir sent les fraises, plus fort. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le loquet garde un fil rouge, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3498,7 +3498,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le loquet garde un fil rouge.</t>
+narrateur|Le loquet garde un fil rouge, minuscule.</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr">
@@ -3530,17 +3530,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. La paille a failli tout plier. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. La paille recouvrait le col, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. La paille a failli tout plier. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. La paille recouvrait le col, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. La paille a failli tout plier. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. Un grain de sable reste au croissant. La paille recouvrait le col, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3697,7 +3697,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Un grain de sable reste au croissant.
-narrateur|La paille a failli tout plier.
+narrateur|La paille recouvrait le col, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -3730,17 +3730,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le chat se recouche, sous la rampe. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le paillasson tient un grain, minuscule.</t>
+          <t>Le chat se recouche, sous la rampe. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un grain reste coincé dans la paille.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le chat se recouche, sous la rampe. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le paillasson tient un grain, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le chat se recouche, sous la rampe. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un grain reste coincé dans la paille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le chat se recouche, sous la rampe. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le paillasson tient un grain, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le chat se recouche, sous la rampe. Chouchou a joué au bac. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un grain reste coincé dans la paille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3889,7 +3889,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le paillasson tient un grain, minuscule.</t>
+narrateur|Un grain reste coincé dans la paille.</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr">
@@ -4312,17 +4312,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le sable a failli tout boire. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le sable buvait la manche, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le sable a failli tout boire. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le sable buvait la manche, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le sable a failli tout boire. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le sable buvait la manche, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4479,7 +4479,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'anse du seau a laissé du sable.
-narrateur|Le sable a failli tout boire.
+narrateur|Le sable buvait la manche, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -4512,17 +4512,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Un grain roule sur une marche. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'anse du seau sèche sous la rampe.</t>
+          <t>Un grain roule sur une marche. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'anse du seau sèche, sous la rampe.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un grain roule sur une marche. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'anse du seau sèche sous la rampe.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un grain roule sur une marche. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'anse du seau sèche, sous la rampe.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un grain roule sur une marche. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'anse du seau sèche sous la rampe.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un grain roule sur une marche. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'anse du seau sèche, sous la rampe.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4671,7 +4671,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|L'anse du seau sèche sous la rampe.</t>
+narrateur|L'anse du seau sèche, sous la rampe.</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr">
@@ -4703,17 +4703,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. L'anse a failli tout tirer. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. L'anse tirait trop, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. L'anse a failli tout tirer. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. L'anse tirait trop, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. L'anse a failli tout tirer. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. L'anse tirait trop, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4870,7 +4870,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'anse du seau a laissé du sable.
-narrateur|L'anse a failli tout tirer.
+narrateur|L'anse tirait trop, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -4903,17 +4903,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le seau pose son ombre au bois. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise roule près du pain.</t>
+          <t>Le seau pose son ombre au bois. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise roule près du pain tiède.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau pose son ombre au bois. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise roule près du pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau pose son ombre au bois. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise roule près du pain tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau pose son ombre au bois. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise roule près du pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau pose son ombre au bois. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise roule près du pain tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -5062,7 +5062,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Une fraise roule près du pain.</t>
+narrateur|Une fraise roule près du pain tiède.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr">
@@ -5094,17 +5094,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le seuil a failli tout garder. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le seuil gardait le pli, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le seuil a failli tout garder. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le seuil gardait le pli, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le seuil a failli tout garder. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'anse du seau a laissé du sable. Le seuil gardait le pli, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5261,7 +5261,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'anse du seau a laissé du sable.
-narrateur|Le seuil a failli tout garder.
+narrateur|Le seuil gardait le pli, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -5294,17 +5294,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Le panier de fraises attend, ouvert. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau pose son ombre au seuil.</t>
+          <t>Le panier de fraises attend, ouvert. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'ombre du seau s'endort au seuil.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le panier de fraises attend, ouvert. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau pose son ombre au seuil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le panier de fraises attend, ouvert. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'ombre du seau s'endort au seuil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le panier de fraises attend, ouvert. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau pose son ombre au seuil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le panier de fraises attend, ouvert. Chouchou a joué au bac. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'ombre du seau s'endort au seuil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5453,7 +5453,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le seau pose son ombre au seuil.</t>
+narrateur|L'ombre du seau s'endort au seuil.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr">
@@ -5876,17 +5876,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le doudou a failli tout cacher. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le doudou cachait le rouge, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le doudou a failli tout cacher. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le doudou cachait le rouge, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le doudou a failli tout cacher. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le doudou cachait le rouge, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -6043,7 +6043,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'oreille du doudou a du sable.
-narrateur|Le doudou a failli tout cacher.
+narrateur|Le doudou cachait le rouge, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -6076,17 +6076,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>L'oreille du doudou dépasse du couloir. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'oreille du doudou veille, au bois.</t>
+          <t>L'oreille du doudou dépasse du couloir. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Du sable reste dans l'oreille du doudou.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille du doudou dépasse du couloir. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'oreille du doudou veille, au bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille du doudou dépasse du couloir. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Du sable reste dans l'oreille du doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille du doudou dépasse du couloir. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'oreille du doudou veille, au bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille du doudou dépasse du couloir. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Du sable reste dans l'oreille du doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6235,7 +6235,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|L'oreille du doudou veille, au bois.</t>
+narrateur|Du sable reste dans l'oreille du doudou.</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr">
@@ -6267,17 +6267,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le fer a failli tout mordre. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le fer mordait la manche, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le fer a failli tout mordre. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le fer mordait la manche, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le fer a failli tout mordre. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le fer mordait la manche, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6434,7 +6434,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'oreille du doudou a du sable.
-narrateur|Le fer a failli tout mordre.
+narrateur|Le fer mordait la manche, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -6467,17 +6467,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Un fil du doudou pend près des clés. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un fil gris pend près des clés.</t>
+          <t>Un fil du doudou pend près des clés. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près des clés, un fil gris pend.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un fil du doudou pend près des clés. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un fil gris pend près des clés.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un fil du doudou pend près des clés. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près des clés, un fil gris pend.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un fil du doudou pend près des clés. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un fil gris pend près des clés.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un fil du doudou pend près des clés. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près des clés, un fil gris pend.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6626,7 +6626,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Un fil gris pend près des clés.</t>
+narrateur|Près des clés, un fil gris pend.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr">
@@ -6658,17 +6658,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le pli a failli tout perdre. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le pli se refermait, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le pli a failli tout perdre. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le pli se refermait, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le pli a failli tout perdre. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le bac, croissant en main. On va au crochet, maintenant. L'oreille du doudou a du sable. Le pli se refermait, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6825,7 +6825,7 @@
 narrateur|On quitte le bac, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'oreille du doudou a du sable.
-narrateur|Le pli a failli tout perdre.
+narrateur|Le pli se refermait, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -6858,17 +6858,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Le doudou sent le sable, au bois. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou garde le sable, au col.</t>
+          <t>Le doudou sent le sable, au bois. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au col, un grain de sable brille.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou sent le sable, au bois. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou garde le sable, au col.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou sent le sable, au bois. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au col, un grain de sable brille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou sent le sable, au bois. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou garde le sable, au col.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou sent le sable, au bois. Chouchou a joué au bac. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au col, un grain de sable brille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -7017,7 +7017,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le doudou garde le sable, au col.</t>
+narrateur|Au col, un grain de sable brille.</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr">
@@ -8199,17 +8199,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. La feuille a failli tout couvrir. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Une feuille couvrait le col, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. La feuille a failli tout couvrir. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Une feuille couvrait le col, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. La feuille a failli tout couvrir. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Une feuille couvrait le col, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8366,7 +8366,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une feuille du toboggan reste au tissu.
-narrateur|La feuille a failli tout couvrir.
+narrateur|Une feuille couvrait le col, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -8399,17 +8399,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Une feuille sèche sur le banc, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une feuille sèche, loin du croissant.</t>
+          <t>Une feuille sèche sur le banc, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une feuille sèche, collée au croissant.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une feuille sèche sur le banc, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une feuille sèche, loin du croissant.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une feuille sèche sur le banc, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une feuille sèche, collée au croissant.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une feuille sèche sur le banc, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une feuille sèche, loin du croissant.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une feuille sèche sur le banc, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une feuille sèche, collée au croissant.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8558,7 +8558,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Une feuille sèche, loin du croissant.</t>
+narrateur|Une feuille sèche, collée au croissant.</t>
         </is>
       </c>
       <c r="AX39" t="inlineStr">
@@ -8590,17 +8590,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le métal a failli tout glisser. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le métal glissait trop, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le métal a failli tout glisser. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le métal glissait trop, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le métal a failli tout glisser. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le métal glissait trop, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8757,7 +8757,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une feuille du toboggan reste au tissu.
-narrateur|Le métal a failli tout glisser.
+narrateur|Le métal glissait trop, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -8790,17 +8790,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le métal du toboggan se tait, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le métal se tait, loin du col.</t>
+          <t>Le métal du toboggan se tait, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin du col, le métal se tait.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le métal du toboggan se tait, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le métal se tait, loin du col.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le métal du toboggan se tait, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin du col, le métal se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le métal du toboggan se tait, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le métal se tait, loin du col.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le métal du toboggan se tait, loin. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin du col, le métal se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8949,7 +8949,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le métal se tait, loin du col.</t>
+narrateur|Loin du col, le métal se tait.</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr">
@@ -8981,17 +8981,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le bord a failli tout plier. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le bord pliait le tissu, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le bord a failli tout plier. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le bord pliait le tissu, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le bord a failli tout plier. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille du toboggan reste au tissu. Le bord pliait le tissu, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -9148,7 +9148,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une feuille du toboggan reste au tissu.
-narrateur|Le bord a failli tout plier.
+narrateur|Le bord pliait le tissu, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -9181,17 +9181,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Un pas sur la rampe, puis plus. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un pas s'éteint, sur le bois.</t>
+          <t>Un pas sur la rampe, puis plus. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur le bois, un pas s'éteint.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un pas sur la rampe, puis plus. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un pas s'éteint, sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un pas sur la rampe, puis plus. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur le bois, un pas s'éteint.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un pas sur la rampe, puis plus. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un pas s'éteint, sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un pas sur la rampe, puis plus. Chouchou a joué au toboggan. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur le bois, un pas s'éteint.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9340,7 +9340,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Un pas s'éteint, sur le bois.</t>
+narrateur|Sur le bois, un pas s'éteint.</t>
         </is>
       </c>
       <c r="AX43" t="inlineStr">
@@ -9763,17 +9763,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. L'eau a failli tout mentir. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. L'eau mentait, une seconde de trop. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. L'eau a failli tout mentir. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. L'eau mentait, une seconde de trop. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. L'eau a failli tout mentir. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. L'eau mentait, une seconde de trop. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9930,7 +9930,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une goutte du seau sèche au croissant.
-narrateur|L'eau a failli tout mentir.
+narrateur|L'eau mentait, une seconde de trop.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -9963,17 +9963,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Le seau penche, sous la rampe. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau penche, vide, sous la rampe.</t>
+          <t>Le seau penche, sous la rampe. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sous la rampe, le seau penche, vide.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau penche, sous la rampe. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau penche, vide, sous la rampe.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau penche, sous la rampe. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sous la rampe, le seau penche, vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau penche, sous la rampe. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau penche, vide, sous la rampe.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau penche, sous la rampe. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sous la rampe, le seau penche, vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -10122,7 +10122,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le seau penche, vide, sous la rampe.</t>
+narrateur|Sous la rampe, le seau penche, vide.</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr">
@@ -10154,17 +10154,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Le seau a failli tout verser. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Le seau versait trop, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Le seau a failli tout verser. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Le seau versait trop, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Le seau a failli tout verser. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Le seau versait trop, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10321,7 +10321,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une goutte du seau sèche au croissant.
-narrateur|Le seau a failli tout verser.
+narrateur|Le seau versait trop, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -10354,17 +10354,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le criiic du portail s'arrête. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le criiic du portail s'endort.</t>
+          <t>Le criiic du portail s'arrête. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le criiic du portail s'endort, loin.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le criiic du portail s'arrête. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le criiic du portail s'endort.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le criiic du portail s'arrête. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le criiic du portail s'endort, loin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le criiic du portail s'arrête. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le criiic du portail s'endort.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le criiic du portail s'arrête. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le criiic du portail s'endort, loin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10513,7 +10513,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le criiic du portail s'endort.</t>
+narrateur|Le criiic du portail s'endort, loin.</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr">
@@ -10545,17 +10545,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. La goutte a failli tout cacher. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Une goutte cachait le croissant, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. La goutte a failli tout cacher. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Une goutte cachait le croissant, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. La goutte a failli tout cacher. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une goutte du seau sèche au croissant. Une goutte cachait le croissant, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10712,7 +10712,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une goutte du seau sèche au croissant.
-narrateur|La goutte a failli tout cacher.
+narrateur|Une goutte cachait le croissant, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -10745,17 +10745,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>La rampe du toboggan reste loin. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. La rampe du toboggan reste muette.</t>
+          <t>La rampe du toboggan reste loin. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin d'ici, la rampe reste muette.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rampe du toboggan reste loin. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. La rampe du toboggan reste muette.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La rampe du toboggan reste loin. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin d'ici, la rampe reste muette.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rampe du toboggan reste loin. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. La rampe du toboggan reste muette.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La rampe du toboggan reste loin. Chouchou a joué au toboggan. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin d'ici, la rampe reste muette.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10904,7 +10904,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|La rampe du toboggan reste muette.</t>
+narrateur|Loin d'ici, la rampe reste muette.</t>
         </is>
       </c>
       <c r="AX51" t="inlineStr">
@@ -11327,17 +11327,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. L'oreille a failli tout prendre. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. L'oreille prenait la place, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. L'oreille a failli tout prendre. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. L'oreille prenait la place, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. L'oreille a failli tout prendre. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. L'oreille prenait la place, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11494,7 +11494,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une feuille reste sur le doudou.
-narrateur|L'oreille a failli tout prendre.
+narrateur|L'oreille prenait la place, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -11527,17 +11527,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>L'oreille molle dépasse du banc. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'oreille molle dépasse, près du banc.</t>
+          <t>L'oreille molle dépasse du banc. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près du banc, une oreille molle veille.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille molle dépasse du banc. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'oreille molle dépasse, près du banc.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille molle dépasse du banc. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près du banc, une oreille molle veille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille molle dépasse du banc. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. L'oreille molle dépasse, près du banc.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille molle dépasse du banc. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près du banc, une oreille molle veille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11686,7 +11686,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|L'oreille molle dépasse, près du banc.</t>
+narrateur|Près du banc, une oreille molle veille.</t>
         </is>
       </c>
       <c r="AX55" t="inlineStr">
@@ -11718,17 +11718,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. Le doudou a failli tout tromper. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. Le doudou trompait l'œil, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. Le doudou a failli tout tromper. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. Le doudou trompait l'œil, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. Le doudou a failli tout tromper. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. Le doudou trompait l'œil, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11885,7 +11885,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une feuille reste sur le doudou.
-narrateur|Le doudou a failli tout tromper.
+narrateur|Le doudou trompait l'œil, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -11918,17 +11918,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a vu le métal, depuis le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou a le métal dans l'oreille.</t>
+          <t>Le doudou a vu le métal, depuis le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans l'oreille, un peu de métal froid.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a vu le métal, depuis le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou a le métal dans l'oreille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a vu le métal, depuis le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans l'oreille, un peu de métal froid.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a vu le métal, depuis le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou a le métal dans l'oreille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a vu le métal, depuis le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans l'oreille, un peu de métal froid.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -12077,7 +12077,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le doudou a le métal dans l'oreille.</t>
+narrateur|Dans l'oreille, un peu de métal froid.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
@@ -12109,17 +12109,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. La feuille a failli tout coller. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. La feuille collait trop, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. La feuille a failli tout coller. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. La feuille collait trop, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. La feuille a failli tout coller. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte le toboggan, croissant en main. On va au crochet, maintenant. Une feuille reste sur le doudou. La feuille collait trop, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -12276,7 +12276,7 @@
 narrateur|On quitte le toboggan, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Une feuille reste sur le doudou.
-narrateur|La feuille a failli tout coller.
+narrateur|La feuille collait trop, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -12309,17 +12309,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Un rayon a bougé, sur le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un rayon a quitté le bois.</t>
+          <t>Un rayon a bougé, sur le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur le bois, le rayon a bougé.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un rayon a bougé, sur le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un rayon a quitté le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un rayon a bougé, sur le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur le bois, le rayon a bougé.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un rayon a bougé, sur le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Un rayon a quitté le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un rayon a bougé, sur le bois. Chouchou a joué au toboggan. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur le bois, le rayon a bougé.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12468,7 +12468,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Un rayon a quitté le bois.</t>
+narrateur|Sur le bois, le rayon a bougé.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr">
@@ -13650,17 +13650,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. La corde a failli tout tenir. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. La corde tenait la manche, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. La corde a failli tout tenir. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. La corde tenait la manche, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. La corde a failli tout tenir. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle cale le ballon sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. La corde tenait la manche, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13817,7 +13817,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Un brin de corde reste au croissant.
-narrateur|La corde a failli tout tenir.
+narrateur|La corde tenait la manche, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -13850,17 +13850,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le ballon s'endort près de l'escalier. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le ballon s'endort, près du cric.</t>
+          <t>Le ballon s'endort près de l'escalier. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près du cric, le ballon s'endort.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le ballon s'endort près de l'escalier. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le ballon s'endort, près du cric.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le ballon s'endort près de l'escalier. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près du cric, le ballon s'endort.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le ballon s'endort près de l'escalier. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le ballon s'endort, près du cric.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le ballon s'endort près de l'escalier. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près du cric, le ballon s'endort.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -14009,7 +14009,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le ballon s'endort, près du cric.</t>
+narrateur|Près du cric, le ballon s'endort.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr">
@@ -14041,17 +14041,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. Le cling a failli tout couvrir. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. Un cling couvrait le croissant, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. Le cling a failli tout couvrir. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. Un cling couvrait le croissant, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. Le cling a failli tout couvrir. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle cale le ballon contre le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. Un cling couvrait le croissant, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -14208,7 +14208,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Un brin de corde reste au croissant.
-narrateur|Le cling a failli tout couvrir.
+narrateur|Un cling couvrait le croissant, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -14241,17 +14241,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>La corde ne fait plus cling. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. La corde se tait, loin du col.</t>
+          <t>La corde ne fait plus cling. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin du col, la corde se tait.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La corde ne fait plus cling. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. La corde se tait, loin du col.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La corde ne fait plus cling. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin du col, la corde se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La corde ne fait plus cling. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. La corde se tait, loin du col.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La corde ne fait plus cling. Chouchou a joué aux cordes. Elle a choisi le ballon, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Loin du col, la corde se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -14400,7 +14400,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|La corde se tait, loin du col.</t>
+narrateur|Loin du col, la corde se tait.</t>
         </is>
       </c>
       <c r="AX69" t="inlineStr">
@@ -14432,17 +14432,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. L'herbe a failli tout cacher. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. L'herbe cachait le col, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. L'herbe a failli tout cacher. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. L'herbe cachait le col, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. L'herbe a failli tout cacher. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle cale le ballon sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le ballon vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Un brin de corde reste au croissant. L'herbe cachait le col, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14599,7 +14599,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Un brin de corde reste au croissant.
-narrateur|L'herbe a failli tout cacher.
+narrateur|L'herbe cachait le col, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -15214,17 +15214,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le seau a failli tout peser. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le seau pesait trop, une seconde. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le seau a failli tout peser. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le seau pesait trop, une seconde. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le seau a failli tout peser. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse l'anse sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le seau pesait trop, une seconde. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -15381,7 +15381,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'anse a senti la corde, froide.
-narrateur|Le seau a failli tout peser.
+narrateur|Le seau pesait trop, une seconde.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -15414,17 +15414,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Le seau pose son ombre sur la marche. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau pose son ombre, sur la marche.</t>
+          <t>Le seau pose son ombre sur la marche. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur la marche, l'ombre du seau dort.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau pose son ombre sur la marche. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau pose son ombre, sur la marche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau pose son ombre sur la marche. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur la marche, l'ombre du seau dort.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau pose son ombre sur la marche. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le seau pose son ombre, sur la marche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau pose son ombre sur la marche. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Sur la marche, l'ombre du seau dort.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15573,7 +15573,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le seau pose son ombre, sur la marche.</t>
+narrateur|Sur la marche, l'ombre du seau dort.</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr">
@@ -15605,17 +15605,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. La corde a failli tout mentir. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. La corde mentait, une seconde de trop. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. La corde a failli tout mentir. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. La corde mentait, une seconde de trop. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. La corde a failli tout mentir. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse l'anse sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. La corde mentait, une seconde de trop. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15772,7 +15772,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'anse a senti la corde, froide.
-narrateur|La corde a failli tout mentir.
+narrateur|La corde mentait, une seconde de trop.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -15805,17 +15805,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le pain tiède attend, sur la table. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le pain tiède attend, près des fraises.</t>
+          <t>Le pain tiède attend, sur la table. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près des fraises, le pain attend.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le pain tiède attend, sur la table. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le pain tiède attend, près des fraises.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le pain tiède attend, sur la table. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près des fraises, le pain attend.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le pain tiède attend, sur la table. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le pain tiède attend, près des fraises.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le pain tiède attend, sur la table. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Près des fraises, le pain attend.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15964,7 +15964,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le pain tiède attend, près des fraises.</t>
+narrateur|Près des fraises, le pain attend.</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr">
@@ -15996,17 +15996,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le pied nu a failli tout perdre. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le pied nu manquait le bord, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le pied nu a failli tout perdre. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le pied nu manquait le bord, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le pied nu a failli tout perdre. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse l'anse sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le seau vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. L'anse a senti la corde, froide. Le pied nu manquait le bord, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -16163,7 +16163,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|L'anse a senti la corde, froide.
-narrateur|Le pied nu a failli tout perdre.
+narrateur|Le pied nu manquait le bord, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -16196,17 +16196,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Les clés de papa restent dans la coupelle. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Les clés restent dans la coupelle.</t>
+          <t>Les clés de papa restent dans la coupelle. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans la coupelle, les clés se taisent.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les clés de papa restent dans la coupelle. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Les clés restent dans la coupelle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les clés de papa restent dans la coupelle. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans la coupelle, les clés se taisent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les clés de papa restent dans la coupelle. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Les clés restent dans la coupelle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les clés de papa restent dans la coupelle. Chouchou a joué aux cordes. Elle a choisi le seau, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans la coupelle, les clés se taisent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -16355,7 +16355,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Les clés restent dans la coupelle.</t>
+narrateur|Dans la coupelle, les clés se taisent.</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr">
@@ -16778,17 +16778,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le siège a failli tout confondre. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le croissant de cuivre brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le siège mélangeait les dos, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le siège a failli tout confondre. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le siège mélangeait les dos, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le siège a failli tout confondre. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le banc. Le bois des lattes est chaud, un peu. Il est dessous, je le vois ! Elle tire la manche, trop vite. Le tissu se coince entre deux lattes. Il tient, entre les lattes ! Le sourire de Chouchou disparaît. Envie et peur se bousculent, dans sa poitrine. Papa s'accroupit, à sa hauteur. Tu regardes, ou tu tires ? Je ne fonce pas. Elle écoute le bois, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, minuscule. La manche avance, puis s'arrête. Elle glisse le doudou sous la latte. Je soulève la latte, sans tirer. La manche se libère, lente, pleine. Tu l'as, sans forcer. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le siège mélangeait les dos, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16945,7 +16945,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Le doudou a l'odeur de l'herbe.
-narrateur|Le siège a failli tout confondre.
+narrateur|Le siège mélangeait les dos, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -16978,17 +16978,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a l'odeur de l'herbe. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou garde l'herbe, au chaud.</t>
+          <t>Le doudou a l'odeur de l'herbe. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au chaud, le doudou sent l'herbe.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a l'odeur de l'herbe. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou garde l'herbe, au chaud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a l'odeur de l'herbe. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au chaud, le doudou sent l'herbe.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a l'odeur de l'herbe. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le doudou garde l'herbe, au chaud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a l'odeur de l'herbe. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le banc. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Où s'était-il caché, sous le banc ? Sous les lattes, avec le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au chaud, le doudou sent l'herbe.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -17137,7 +17137,7 @@
 enfant-f|Sous les lattes, avec le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le doudou garde l'herbe, au chaud.</t>
+narrateur|Au chaud, le doudou sent l'herbe.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -17169,17 +17169,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le dos flou a failli tout prendre. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le croissant de cuivre clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Un dos flou prenait la place, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le dos flou a failli tout prendre. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Un dos flou prenait la place, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Le dos flou a failli tout prendre. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le portail. Le loquet est froid, un peu rêche. Il est accroché, je le vois ! Elle tire la manche, trop vite. Le tissu s'enroule autour du loquet. Le loquet le mange ! Ses épaules baissent, près du fer. Dans sa poitrine, ça serre, trop fort. Maman s'accroupit, à sa hauteur. Tu forces, ou tu regardes ? J'attends, je regarde. Elle écoute le fer, puis le col. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; clignote, minuscule. Le col glisse, puis se bloque. Elle glisse le doudou sous le loquet. Je soulève le loquet, sans tirer. La manche se libère, lente, froide. Il est à toi, maintenant. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. Un dos flou prenait la place, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -17336,7 +17336,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Le doudou a l'odeur de l'herbe.
-narrateur|Le dos flou a failli tout prendre.
+narrateur|Un dos flou prenait la place, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -17369,17 +17369,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Une fraise rentre dans le panier. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise rentre, rouge, dans le panier.</t>
+          <t>Une fraise rentre dans le panier. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans le panier, une fraise rentre.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une fraise rentre dans le panier. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise rentre, rouge, dans le panier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une fraise rentre dans le panier. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans le panier, une fraise rentre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une fraise rentre dans le panier. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Une fraise rentre, rouge, dans le panier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une fraise rentre dans le panier. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le portail. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait pris, au loquet ? Le loquet, et le croissant. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Dans le panier, une fraise rentre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -17528,7 +17528,7 @@
 enfant-f|Le loquet, et le croissant.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Une fraise rentre, rouge, dans le panier.</t>
+narrateur|Dans le panier, une fraise rentre.</t>
         </is>
       </c>
       <c r="AX85" t="inlineStr">
@@ -17560,17 +17560,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. L'odeur a failli tout perdre. Voilà le manteau, au coin des crochets.</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le croissant de cuivre brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. L'odeur égarait la main, presque. Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. L'odeur a failli tout perdre. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis level="moderate"&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. L'odeur égarait la main, presque. Voilà le manteau, au coin des crochets.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. L'odeur a failli tout perdre. Voilà le manteau, au coin des crochets. [pause]</t>
+          <t>Le croissant court vers le paillasson. La paille est rêche, couleur d'herbe. Il est plié, je le vois ! Elle tire le pli, trop vite. Le tissu se coince sous le seuil. Le seuil le garde ! Chouchou fixe le pli, sans bouger. L'envie de tirer lui pique les doigts. Papa s'accroupit, près du paillasson. Tu vois le croissant, où ? Je cherche, sans tirer. Elle écarte la paille, lente. Le &lt;emphasis&gt;croissant de cuivre&lt;/emphasis&gt; brille, sous le bord. Un pli cède, puis refuse. Elle glisse le doudou sous le bord. Je soulève le bord, sans tirer. La manche se libère, lente, rêche. Tu l'as repris, Chouchou. Chouchou serre le manteau, fière. Le doudou vient aussi, près d'elle. On quitte les cordes, croissant en main. On va au crochet, maintenant. Le doudou a l'odeur de l'herbe. L'odeur égarait la main, presque. Voilà le manteau, au coin des crochets. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17727,7 +17727,7 @@
 narrateur|On quitte les cordes, croissant en main.
 enfant-f|On va au crochet, maintenant.
 narrateur|Le doudou a l'odeur de l'herbe.
-narrateur|L'odeur a failli tout perdre.
+narrateur|L'odeur égarait la main, presque.
 narrateur|Voilà le manteau, au coin des crochets.</t>
         </is>
       </c>
@@ -17760,17 +17760,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Le couloir retrouve son cric, unique. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le croissant de cuivre se tait, au crochet.</t>
+          <t>Le couloir retrouve son cric, unique. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le croissant l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au crochet, le croissant de cuivre se tait.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couloir retrouve son cric, unique. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le croissant de cuivre se tait, au crochet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le couloir retrouve son cric, unique. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis level="moderate"&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au crochet, le croissant de cuivre se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couloir retrouve son cric, unique. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Le croissant de cuivre se tait, au crochet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le couloir retrouve son cric, unique. Chouchou a joué aux cordes. Elle a choisi le doudou, pour le jeu. Le &lt;emphasis&gt;croissant&lt;/emphasis&gt; l'a menée vers le paillasson. Voilà le manteau rouge, sur la rampe. Au col, le croissant de cuivre brille. Il est rentré, avec sa trace. Qui l'avait plié, sur la paille ? Le paillasson, tout plat. Les fraises nous attendent, maintenant. Je croque, elle est sucrée. Au crochet, le croissant de cuivre se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17919,7 +17919,7 @@
 enfant-f|Le paillasson, tout plat.
 maman|Les fraises nous attendent, maintenant.
 enfant-f|Je croque, elle est sucrée.
-narrateur|Le croissant de cuivre se tait, au crochet.</t>
+narrateur|Au crochet, le croissant de cuivre se tait.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr">
@@ -17945,7 +17945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -18058,6 +18058,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>